<commit_message>
new figures for habitat and methods
</commit_message>
<xml_diff>
--- a/data/data_extraction/data_extraction_final.xlsx
+++ b/data/data_extraction/data_extraction_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j_stee03\Uni\takeoff\data\data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D56DBE8-A2B7-4DBA-9A16-C84CC67AC3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D84B6B5-4ABB-4244-A387-995A3899F5E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45600" yWindow="0" windowWidth="21600" windowHeight="15585" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12929" uniqueCount="2410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12930" uniqueCount="2411">
   <si>
     <t>Metadata</t>
   </si>
@@ -7295,6 +7295,9 @@
   </si>
   <si>
     <t>10.5281/zenodo.5337058</t>
+  </si>
+  <si>
+    <t>0,5837</t>
   </si>
 </sst>
 </file>
@@ -7726,16 +7729,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -8058,15 +8061,15 @@
       <c r="H1" s="126"/>
       <c r="I1" s="126"/>
       <c r="J1" s="126"/>
-      <c r="K1" s="127" t="s">
+      <c r="K1" s="128" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="127"/>
-      <c r="N1" s="127"/>
-      <c r="O1" s="127"/>
-      <c r="P1" s="127"/>
-      <c r="Q1" s="127"/>
+      <c r="L1" s="128"/>
+      <c r="M1" s="128"/>
+      <c r="N1" s="128"/>
+      <c r="O1" s="128"/>
+      <c r="P1" s="128"/>
+      <c r="Q1" s="128"/>
       <c r="R1" s="126" t="s">
         <v>2</v>
       </c>
@@ -8078,30 +8081,30 @@
       <c r="X1" s="126"/>
       <c r="Y1" s="126"/>
       <c r="Z1" s="126"/>
-      <c r="AA1" s="127" t="s">
+      <c r="AA1" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="AB1" s="127"/>
-      <c r="AC1" s="127"/>
-      <c r="AD1" s="127"/>
-      <c r="AE1" s="127" t="s">
+      <c r="AB1" s="128"/>
+      <c r="AC1" s="128"/>
+      <c r="AD1" s="128"/>
+      <c r="AE1" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="AF1" s="127"/>
-      <c r="AG1" s="127"/>
-      <c r="AH1" s="127"/>
-      <c r="AI1" s="125" t="s">
+      <c r="AF1" s="128"/>
+      <c r="AG1" s="128"/>
+      <c r="AH1" s="128"/>
+      <c r="AI1" s="127" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="125"/>
-      <c r="AK1" s="125"/>
-      <c r="AL1" s="125"/>
-      <c r="AM1" s="125"/>
-      <c r="AN1" s="128" t="s">
+      <c r="AJ1" s="127"/>
+      <c r="AK1" s="127"/>
+      <c r="AL1" s="127"/>
+      <c r="AM1" s="127"/>
+      <c r="AN1" s="125" t="s">
         <v>6</v>
       </c>
       <c r="AO1" s="126"/>
-      <c r="AP1" s="125"/>
+      <c r="AP1" s="127"/>
       <c r="AR1"/>
     </row>
     <row r="2" spans="1:44" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -24897,7 +24900,7 @@
         <v>71</v>
       </c>
       <c r="AM192" s="46">
-        <v>92.7</v>
+        <v>0.92700000000000005</v>
       </c>
       <c r="AN192" s="30" t="s">
         <v>54</v>
@@ -55235,8 +55238,8 @@
       <c r="AL593" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="AM593" s="90">
-        <v>58.37</v>
+      <c r="AM593" s="90" t="s">
+        <v>2410</v>
       </c>
       <c r="AN593" s="17"/>
       <c r="AO593" s="17"/>
@@ -66629,8 +66632,8 @@
     <row r="734" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="Y1:Y734" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:AQ734">
-    <sortCondition ref="A1:A734"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:AQ735">
+    <sortCondition ref="A1:A735"/>
   </sortState>
   <mergeCells count="7">
     <mergeCell ref="AN1:AP1"/>

</xml_diff>